<commit_message>
Taz and landuse stat updated
TAZ and landuse stat were updated. created new landuse tab
</commit_message>
<xml_diff>
--- a/docs/other/xlsx/LandUseStat.xlsx
+++ b/docs/other/xlsx/LandUseStat.xlsx
@@ -5,27 +5,27 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Employee\DAP\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MRM\docs\other\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3391604D-7CFD-4D67-B3CF-86722A8845DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D10C655-841E-4426-90FD-7E41737E4E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A1C30AB-F8D3-4A56-9DBB-1BE20D40B24B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="12" xr2:uid="{3A1C30AB-F8D3-4A56-9DBB-1BE20D40B24B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Anson3.1" sheetId="13" r:id="rId1"/>
-    <sheet name="Cabarrus3.2" sheetId="1" r:id="rId2"/>
-    <sheet name="Rowan3.3" sheetId="2" r:id="rId3"/>
-    <sheet name="Iredell3.4" sheetId="3" r:id="rId4"/>
-    <sheet name="Mecklenburg3.5" sheetId="4" r:id="rId5"/>
-    <sheet name="Union3.6" sheetId="5" r:id="rId6"/>
-    <sheet name="Stanly3.7" sheetId="6" r:id="rId7"/>
-    <sheet name="Cleveland3.8" sheetId="7" r:id="rId8"/>
-    <sheet name="Gaston3.9" sheetId="8" r:id="rId9"/>
-    <sheet name="Lincoln3.10" sheetId="9" r:id="rId10"/>
-    <sheet name="Lancaster3.11" sheetId="10" r:id="rId11"/>
-    <sheet name="York3.12" sheetId="11" r:id="rId12"/>
-    <sheet name="Catawba3.13" sheetId="12" r:id="rId13"/>
+    <sheet name="Anson" sheetId="13" r:id="rId1"/>
+    <sheet name="Cabarrus" sheetId="1" r:id="rId2"/>
+    <sheet name="Rowan" sheetId="2" r:id="rId3"/>
+    <sheet name="Iredell" sheetId="3" r:id="rId4"/>
+    <sheet name="Mecklenburg" sheetId="4" r:id="rId5"/>
+    <sheet name="Union" sheetId="5" r:id="rId6"/>
+    <sheet name="Stanly" sheetId="6" r:id="rId7"/>
+    <sheet name="Cleveland" sheetId="7" r:id="rId8"/>
+    <sheet name="Gaston" sheetId="8" r:id="rId9"/>
+    <sheet name="Lincoln" sheetId="9" r:id="rId10"/>
+    <sheet name="Lancaster" sheetId="10" r:id="rId11"/>
+    <sheet name="York" sheetId="11" r:id="rId12"/>
+    <sheet name="Catawba" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>